<commit_message>
Add 4-part deck: level overview, table 1 (status), table 2 (supplement), possible methods; refresh report tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GquJWFp9qb794TPiMPAuJn
</commit_message>
<xml_diff>
--- a/docs/字段现状与补充方式.xlsx
+++ b/docs/字段现状与补充方式.xlsx
@@ -464,6 +464,9 @@
     <t>座舱视频</t>
   </si>
   <si>
+    <t>路段表</t>
+  </si>
+  <si>
     <t>接管时刻</t>
   </si>
   <si>
@@ -494,16 +497,13 @@
     <t>已有</t>
   </si>
   <si>
+    <t>人工·前视</t>
+  </si>
+  <si>
+    <t>模型·座舱</t>
+  </si>
+  <si>
     <t>人工·座舱</t>
-  </si>
-  <si>
-    <t>人工·前视</t>
-  </si>
-  <si>
-    <t>模型·音轨</t>
-  </si>
-  <si>
-    <t>模型·座舱</t>
   </si>
   <si>
     <t>模型·踏板</t>
@@ -988,10 +988,10 @@
         <v>138</v>
       </c>
       <c r="L3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N3" t="s">
         <v>138</v>
@@ -1164,10 +1164,10 @@
         <v>141</v>
       </c>
       <c r="L7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N7" t="s">
         <v>141</v>
@@ -1187,13 +1187,13 @@
         <v>142</v>
       </c>
       <c r="E8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H8" t="s">
         <v>142</v>
@@ -1275,13 +1275,13 @@
         <v>142</v>
       </c>
       <c r="E10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H10" t="s">
         <v>142</v>
@@ -1319,13 +1319,13 @@
         <v>142</v>
       </c>
       <c r="E11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H11" t="s">
         <v>142</v>
@@ -1334,19 +1334,19 @@
         <v>142</v>
       </c>
       <c r="J11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -1583,13 +1583,13 @@
         <v>142</v>
       </c>
       <c r="E17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H17" t="s">
         <v>142</v>
@@ -1598,10 +1598,10 @@
         <v>142</v>
       </c>
       <c r="J17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L17" t="s">
         <v>142</v>
@@ -1610,7 +1610,7 @@
         <v>142</v>
       </c>
       <c r="N17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -2044,10 +2044,10 @@
         <v>138</v>
       </c>
       <c r="L27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M27" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N27" t="s">
         <v>138</v>
@@ -2903,7 +2903,7 @@
         <v>142</v>
       </c>
       <c r="E47" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F47" t="s">
         <v>138</v>
@@ -2924,10 +2924,10 @@
         <v>138</v>
       </c>
       <c r="L47" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M47" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N47" t="s">
         <v>138</v>
@@ -2947,7 +2947,7 @@
         <v>142</v>
       </c>
       <c r="E48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F48" t="s">
         <v>138</v>
@@ -2968,10 +2968,10 @@
         <v>138</v>
       </c>
       <c r="L48" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M48" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N48" t="s">
         <v>138</v>
@@ -2991,7 +2991,7 @@
         <v>142</v>
       </c>
       <c r="E49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F49" t="s">
         <v>138</v>
@@ -3035,7 +3035,7 @@
         <v>142</v>
       </c>
       <c r="E50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F50" t="s">
         <v>138</v>
@@ -3056,10 +3056,10 @@
         <v>138</v>
       </c>
       <c r="L50" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M50" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N50" t="s">
         <v>138</v>
@@ -3364,13 +3364,13 @@
         <v>138</v>
       </c>
       <c r="L57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M57" t="s">
         <v>138</v>
       </c>
       <c r="N57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -3651,7 +3651,7 @@
         <v>142</v>
       </c>
       <c r="E64" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F64" t="s">
         <v>138</v>
@@ -3695,7 +3695,7 @@
         <v>142</v>
       </c>
       <c r="E65" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F65" t="s">
         <v>138</v>
@@ -4088,10 +4088,10 @@
         <v>135</v>
       </c>
       <c r="D74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="E74" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F74" t="s">
         <v>138</v>
@@ -4100,10 +4100,10 @@
         <v>138</v>
       </c>
       <c r="H74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="I74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="J74" t="s">
         <v>138</v>
@@ -4112,10 +4112,10 @@
         <v>138</v>
       </c>
       <c r="L74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="M74" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="N74" t="s">
         <v>138</v>
@@ -4200,13 +4200,13 @@
         <v>138</v>
       </c>
       <c r="L76" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M76" t="s">
         <v>138</v>
       </c>
       <c r="N76" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -4244,7 +4244,7 @@
         <v>138</v>
       </c>
       <c r="L77" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M77" t="s">
         <v>138</v>
@@ -4288,7 +4288,7 @@
         <v>138</v>
       </c>
       <c r="L78" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M78" t="s">
         <v>138</v>
@@ -4332,7 +4332,7 @@
         <v>138</v>
       </c>
       <c r="L79" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M79" t="s">
         <v>138</v>
@@ -4376,7 +4376,7 @@
         <v>138</v>
       </c>
       <c r="L80" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M80" t="s">
         <v>138</v>
@@ -4420,13 +4420,13 @@
         <v>138</v>
       </c>
       <c r="L81" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M81" t="s">
         <v>138</v>
       </c>
       <c r="N81" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -4464,13 +4464,13 @@
         <v>138</v>
       </c>
       <c r="L82" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M82" t="s">
         <v>138</v>
       </c>
       <c r="N82" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -4508,13 +4508,13 @@
         <v>138</v>
       </c>
       <c r="L83" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M83" t="s">
         <v>138</v>
       </c>
       <c r="N83" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -4552,13 +4552,13 @@
         <v>138</v>
       </c>
       <c r="L84" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M84" t="s">
         <v>138</v>
       </c>
       <c r="N84" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -4596,13 +4596,13 @@
         <v>138</v>
       </c>
       <c r="L85" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M85" t="s">
         <v>138</v>
       </c>
       <c r="N85" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -4640,10 +4640,10 @@
         <v>138</v>
       </c>
       <c r="L86" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M86" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N86" t="s">
         <v>138</v>
@@ -4684,7 +4684,7 @@
         <v>138</v>
       </c>
       <c r="L87" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M87" t="s">
         <v>138</v>
@@ -4728,10 +4728,10 @@
         <v>138</v>
       </c>
       <c r="L88" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M88" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="N88" t="s">
         <v>138</v>
@@ -4948,13 +4948,13 @@
         <v>138</v>
       </c>
       <c r="L93" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M93" t="s">
         <v>138</v>
       </c>
       <c r="N93" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -5036,13 +5036,13 @@
         <v>138</v>
       </c>
       <c r="L95" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="M95" t="s">
         <v>138</v>
       </c>
       <c r="N95" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -5364,37 +5364,37 @@
         <v>134</v>
       </c>
       <c r="D103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="N103" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -5411,7 +5411,7 @@
         <v>142</v>
       </c>
       <c r="E104" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F104" t="s">
         <v>138</v>
@@ -5628,25 +5628,25 @@
         <v>134</v>
       </c>
       <c r="D109" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E109" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F109" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G109" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H109" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I109" t="s">
         <v>138</v>
       </c>
       <c r="J109" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K109" t="s">
         <v>138</v>
@@ -5675,7 +5675,7 @@
         <v>142</v>
       </c>
       <c r="E110" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F110" t="s">
         <v>138</v>
@@ -5814,7 +5814,7 @@
         <v>134</v>
       </c>
       <c r="D2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E2" t="s">
         <v>167</v>
@@ -5826,10 +5826,10 @@
         <v>167</v>
       </c>
       <c r="H2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J2" t="s">
         <v>138</v>
@@ -5882,10 +5882,10 @@
         <v>138</v>
       </c>
       <c r="L3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N3" t="s">
         <v>138</v>
@@ -5902,37 +5902,37 @@
         <v>134</v>
       </c>
       <c r="D4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -5946,37 +5946,37 @@
         <v>134</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -5990,37 +5990,37 @@
         <v>134</v>
       </c>
       <c r="D6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -6034,37 +6034,37 @@
         <v>134</v>
       </c>
       <c r="D7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -6078,22 +6078,22 @@
         <v>134</v>
       </c>
       <c r="D8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J8" t="s">
         <v>138</v>
@@ -6102,10 +6102,10 @@
         <v>138</v>
       </c>
       <c r="L8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N8" t="s">
         <v>138</v>
@@ -6122,37 +6122,37 @@
         <v>135</v>
       </c>
       <c r="D9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -6166,22 +6166,22 @@
         <v>135</v>
       </c>
       <c r="D10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J10" t="s">
         <v>138</v>
@@ -6190,10 +6190,10 @@
         <v>138</v>
       </c>
       <c r="L10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N10" t="s">
         <v>138</v>
@@ -6210,37 +6210,37 @@
         <v>134</v>
       </c>
       <c r="D11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -6254,37 +6254,37 @@
         <v>134</v>
       </c>
       <c r="D12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N12" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -6386,22 +6386,22 @@
         <v>134</v>
       </c>
       <c r="D15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G15" t="s">
         <v>138</v>
       </c>
       <c r="H15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J15" t="s">
         <v>170</v>
@@ -6430,13 +6430,13 @@
         <v>135</v>
       </c>
       <c r="D16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G16" t="s">
         <v>138</v>
@@ -6474,37 +6474,37 @@
         <v>134</v>
       </c>
       <c r="D17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -6518,22 +6518,22 @@
         <v>135</v>
       </c>
       <c r="D18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G18" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J18" t="s">
         <v>138</v>
@@ -6618,10 +6618,10 @@
         <v>138</v>
       </c>
       <c r="H20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J20" t="s">
         <v>138</v>
@@ -6662,10 +6662,10 @@
         <v>138</v>
       </c>
       <c r="H21" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I21" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J21" t="s">
         <v>138</v>
@@ -6694,22 +6694,22 @@
         <v>135</v>
       </c>
       <c r="D22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G22" t="s">
         <v>138</v>
       </c>
       <c r="H22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J22" t="s">
         <v>138</v>
@@ -6738,7 +6738,7 @@
         <v>134</v>
       </c>
       <c r="D23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E23" t="s">
         <v>161</v>
@@ -6750,10 +6750,10 @@
         <v>161</v>
       </c>
       <c r="H23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J23" t="s">
         <v>138</v>
@@ -6782,22 +6782,22 @@
         <v>134</v>
       </c>
       <c r="D24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I24" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J24" t="s">
         <v>138</v>
@@ -6826,22 +6826,22 @@
         <v>134</v>
       </c>
       <c r="D25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I25" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J25" t="s">
         <v>138</v>
@@ -6870,7 +6870,7 @@
         <v>135</v>
       </c>
       <c r="D26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E26" t="s">
         <v>167</v>
@@ -6882,10 +6882,10 @@
         <v>167</v>
       </c>
       <c r="H26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I26" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J26" t="s">
         <v>138</v>
@@ -6938,10 +6938,10 @@
         <v>138</v>
       </c>
       <c r="L27" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M27" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N27" t="s">
         <v>138</v>
@@ -7090,22 +7090,22 @@
         <v>134</v>
       </c>
       <c r="D31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J31" t="s">
         <v>138</v>
@@ -7134,22 +7134,22 @@
         <v>134</v>
       </c>
       <c r="D32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J32" t="s">
         <v>138</v>
@@ -7178,22 +7178,22 @@
         <v>134</v>
       </c>
       <c r="D33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J33" t="s">
         <v>138</v>
@@ -7222,22 +7222,22 @@
         <v>135</v>
       </c>
       <c r="D34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I34" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J34" t="s">
         <v>138</v>
@@ -7266,37 +7266,37 @@
         <v>134</v>
       </c>
       <c r="D35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -7310,22 +7310,22 @@
         <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E36" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F36" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G36" t="s">
         <v>138</v>
       </c>
       <c r="H36" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I36" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J36" t="s">
         <v>138</v>
@@ -7354,16 +7354,16 @@
         <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G37" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H37" t="s">
         <v>138</v>
@@ -7398,16 +7398,16 @@
         <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H38" t="s">
         <v>138</v>
@@ -7442,16 +7442,16 @@
         <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G39" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H39" t="s">
         <v>138</v>
@@ -7486,16 +7486,16 @@
         <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H40" t="s">
         <v>138</v>
@@ -7530,16 +7530,16 @@
         <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G41" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H41" t="s">
         <v>138</v>
@@ -7574,16 +7574,16 @@
         <v>135</v>
       </c>
       <c r="D42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G42" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H42" t="s">
         <v>138</v>
@@ -7618,13 +7618,13 @@
         <v>134</v>
       </c>
       <c r="D43" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E43" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F43" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G43" t="s">
         <v>138</v>
@@ -7662,16 +7662,16 @@
         <v>135</v>
       </c>
       <c r="D44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G44" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H44" t="s">
         <v>138</v>
@@ -7750,16 +7750,16 @@
         <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G46" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H46" t="s">
         <v>138</v>
@@ -7794,10 +7794,10 @@
         <v>134</v>
       </c>
       <c r="D47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F47" t="s">
         <v>164</v>
@@ -7806,10 +7806,10 @@
         <v>138</v>
       </c>
       <c r="H47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J47" t="s">
         <v>138</v>
@@ -7818,10 +7818,10 @@
         <v>138</v>
       </c>
       <c r="L47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N47" t="s">
         <v>138</v>
@@ -7838,10 +7838,10 @@
         <v>134</v>
       </c>
       <c r="D48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F48" t="s">
         <v>164</v>
@@ -7850,10 +7850,10 @@
         <v>138</v>
       </c>
       <c r="H48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J48" t="s">
         <v>138</v>
@@ -7862,10 +7862,10 @@
         <v>138</v>
       </c>
       <c r="L48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M48" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N48" t="s">
         <v>138</v>
@@ -7882,10 +7882,10 @@
         <v>134</v>
       </c>
       <c r="D49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F49" t="s">
         <v>164</v>
@@ -7894,10 +7894,10 @@
         <v>138</v>
       </c>
       <c r="H49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J49" t="s">
         <v>138</v>
@@ -7906,10 +7906,10 @@
         <v>138</v>
       </c>
       <c r="L49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N49" t="s">
         <v>138</v>
@@ -7926,10 +7926,10 @@
         <v>135</v>
       </c>
       <c r="D50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F50" t="s">
         <v>164</v>
@@ -7938,10 +7938,10 @@
         <v>138</v>
       </c>
       <c r="H50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J50" t="s">
         <v>138</v>
@@ -7950,10 +7950,10 @@
         <v>138</v>
       </c>
       <c r="L50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M50" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N50" t="s">
         <v>138</v>
@@ -7970,16 +7970,16 @@
         <v>134</v>
       </c>
       <c r="D51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H51" t="s">
         <v>138</v>
@@ -8014,16 +8014,16 @@
         <v>135</v>
       </c>
       <c r="D52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H52" t="s">
         <v>138</v>
@@ -8258,13 +8258,13 @@
         <v>138</v>
       </c>
       <c r="L57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M57" t="s">
         <v>138</v>
       </c>
       <c r="N57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="58" spans="1:14">
@@ -8322,16 +8322,16 @@
         <v>134</v>
       </c>
       <c r="D59" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E59" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F59" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G59" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H59" t="s">
         <v>138</v>
@@ -8410,16 +8410,16 @@
         <v>134</v>
       </c>
       <c r="D61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G61" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H61" t="s">
         <v>138</v>
@@ -8498,22 +8498,22 @@
         <v>134</v>
       </c>
       <c r="D63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J63" t="s">
         <v>138</v>
@@ -8542,10 +8542,10 @@
         <v>134</v>
       </c>
       <c r="D64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F64" t="s">
         <v>164</v>
@@ -8554,10 +8554,10 @@
         <v>138</v>
       </c>
       <c r="H64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J64" t="s">
         <v>138</v>
@@ -8566,10 +8566,10 @@
         <v>138</v>
       </c>
       <c r="L64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N64" t="s">
         <v>138</v>
@@ -8586,10 +8586,10 @@
         <v>134</v>
       </c>
       <c r="D65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F65" t="s">
         <v>164</v>
@@ -8598,10 +8598,10 @@
         <v>138</v>
       </c>
       <c r="H65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J65" t="s">
         <v>138</v>
@@ -8610,10 +8610,10 @@
         <v>138</v>
       </c>
       <c r="L65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N65" t="s">
         <v>138</v>
@@ -8850,7 +8850,7 @@
         <v>134</v>
       </c>
       <c r="D71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E71" t="s">
         <v>165</v>
@@ -8862,10 +8862,10 @@
         <v>167</v>
       </c>
       <c r="H71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I71" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J71" t="s">
         <v>138</v>
@@ -8982,10 +8982,10 @@
         <v>135</v>
       </c>
       <c r="D74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F74" t="s">
         <v>164</v>
@@ -8994,10 +8994,10 @@
         <v>138</v>
       </c>
       <c r="H74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J74" t="s">
         <v>138</v>
@@ -9006,10 +9006,10 @@
         <v>138</v>
       </c>
       <c r="L74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M74" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N74" t="s">
         <v>138</v>
@@ -9070,7 +9070,7 @@
         <v>134</v>
       </c>
       <c r="D76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E76" t="s">
         <v>164</v>
@@ -9082,10 +9082,10 @@
         <v>138</v>
       </c>
       <c r="H76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J76" t="s">
         <v>169</v>
@@ -9094,13 +9094,13 @@
         <v>138</v>
       </c>
       <c r="L76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M76" t="s">
         <v>138</v>
       </c>
       <c r="N76" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -9138,7 +9138,7 @@
         <v>138</v>
       </c>
       <c r="L77" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M77" t="s">
         <v>138</v>
@@ -9182,7 +9182,7 @@
         <v>138</v>
       </c>
       <c r="L78" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M78" t="s">
         <v>138</v>
@@ -9226,7 +9226,7 @@
         <v>138</v>
       </c>
       <c r="L79" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M79" t="s">
         <v>138</v>
@@ -9270,7 +9270,7 @@
         <v>138</v>
       </c>
       <c r="L80" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M80" t="s">
         <v>138</v>
@@ -9314,13 +9314,13 @@
         <v>138</v>
       </c>
       <c r="L81" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M81" t="s">
         <v>138</v>
       </c>
       <c r="N81" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -9358,13 +9358,13 @@
         <v>138</v>
       </c>
       <c r="L82" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M82" t="s">
         <v>138</v>
       </c>
       <c r="N82" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -9402,13 +9402,13 @@
         <v>138</v>
       </c>
       <c r="L83" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M83" t="s">
         <v>138</v>
       </c>
       <c r="N83" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -9446,13 +9446,13 @@
         <v>138</v>
       </c>
       <c r="L84" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M84" t="s">
         <v>138</v>
       </c>
       <c r="N84" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -9490,13 +9490,13 @@
         <v>138</v>
       </c>
       <c r="L85" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M85" t="s">
         <v>138</v>
       </c>
       <c r="N85" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -9534,10 +9534,10 @@
         <v>138</v>
       </c>
       <c r="L86" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M86" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N86" t="s">
         <v>138</v>
@@ -9578,7 +9578,7 @@
         <v>138</v>
       </c>
       <c r="L87" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M87" t="s">
         <v>138</v>
@@ -9622,10 +9622,10 @@
         <v>138</v>
       </c>
       <c r="L88" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M88" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N88" t="s">
         <v>138</v>
@@ -9730,7 +9730,7 @@
         <v>135</v>
       </c>
       <c r="D91" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E91" t="s">
         <v>164</v>
@@ -9742,10 +9742,10 @@
         <v>138</v>
       </c>
       <c r="H91" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I91" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J91" t="s">
         <v>170</v>
@@ -9842,13 +9842,13 @@
         <v>138</v>
       </c>
       <c r="L93" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M93" t="s">
         <v>165</v>
       </c>
       <c r="N93" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -9930,13 +9930,13 @@
         <v>138</v>
       </c>
       <c r="L95" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M95" t="s">
         <v>138</v>
       </c>
       <c r="N95" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -9950,7 +9950,7 @@
         <v>135</v>
       </c>
       <c r="D96" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E96" t="s">
         <v>168</v>
@@ -9962,10 +9962,10 @@
         <v>168</v>
       </c>
       <c r="H96" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I96" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J96" t="s">
         <v>168</v>
@@ -9994,7 +9994,7 @@
         <v>135</v>
       </c>
       <c r="D97" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E97" t="s">
         <v>166</v>
@@ -10006,10 +10006,10 @@
         <v>166</v>
       </c>
       <c r="H97" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I97" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J97" t="s">
         <v>138</v>
@@ -10258,37 +10258,37 @@
         <v>134</v>
       </c>
       <c r="D103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N103" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -10302,10 +10302,10 @@
         <v>134</v>
       </c>
       <c r="D104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F104" t="s">
         <v>138</v>
@@ -10314,10 +10314,10 @@
         <v>138</v>
       </c>
       <c r="H104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J104" t="s">
         <v>138</v>
@@ -10326,10 +10326,10 @@
         <v>138</v>
       </c>
       <c r="L104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M104" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N104" t="s">
         <v>138</v>
@@ -10346,7 +10346,7 @@
         <v>134</v>
       </c>
       <c r="D105" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E105" t="s">
         <v>167</v>
@@ -10358,10 +10358,10 @@
         <v>167</v>
       </c>
       <c r="H105" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I105" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J105" t="s">
         <v>170</v>
@@ -10522,25 +10522,25 @@
         <v>134</v>
       </c>
       <c r="D109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I109" t="s">
         <v>138</v>
       </c>
       <c r="J109" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K109" t="s">
         <v>138</v>
@@ -10566,10 +10566,10 @@
         <v>135</v>
       </c>
       <c r="D110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F110" t="s">
         <v>164</v>
@@ -10578,10 +10578,10 @@
         <v>138</v>
       </c>
       <c r="H110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="J110" t="s">
         <v>169</v>
@@ -10590,10 +10590,10 @@
         <v>138</v>
       </c>
       <c r="L110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M110" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N110" t="s">
         <v>138</v>

</xml_diff>